<commit_message>
Introduced logs(log4j2) and listeners(ITestListener) into the framework
-> Added log4j2 core, log4j2 api, log4j2 Slf4j2 impl dependency to
pom.xml file
-> Created log4j2 configuration file to store the logs to Console and
file
-> Created LoggerUtility to follow SignletonDesign pattern for creating
one logger object
-> Introduced logs for now: Home Page and BrowserUtility class
-> Created TestListener class implements ITestListener for capturing
when test suite started, test status like pass, fail or skip, when test
suite finished
</commit_message>
<xml_diff>
--- a/testData/loginData.xlsx
+++ b/testData/loginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\SDET with Jatin\Java Module\telit-automation-assignment\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04038F64-E8E3-4450-AFD6-E42F8F8390DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B25E926-52D8-41BF-B7BB-7F58B8ADB530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>emailAddress</t>
   </si>
@@ -38,12 +38,6 @@
   </si>
   <si>
     <t>Pwd@123</t>
-  </si>
-  <si>
-    <t>agchetan18@gmail.com</t>
-  </si>
-  <si>
-    <t>rcb@2026</t>
   </si>
 </sst>
 </file>
@@ -379,7 +373,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" bestFit="1" customWidth="1"/>
@@ -402,20 +396,10 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{54A0116B-3072-46CC-90C9-010F80C7C89F}"/>
     <hyperlink ref="B2" r:id="rId2" xr:uid="{4CFC90D1-FD39-4509-8A12-1B136C93D440}"/>
-    <hyperlink ref="A3" r:id="rId3" xr:uid="{CA6C3426-E82B-477C-A6C8-C2748C3FB23F}"/>
-    <hyperlink ref="B3" r:id="rId4" xr:uid="{AF29C2D8-9000-4B44-90D7-11BBBFD701F1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>